<commit_message>
feat: expansão B3 para 81 empresas + UX dashboard
- CVM_TO_TICKER expandido: 24 → 78 mapeamentos (b3_runner.py)
- CVM_TO_TICKER_CLEAN expandido: 102 → 175 entradas (b3_catalog.py)
- Pipeline B3: 24 → 81 empresas processadas
- Dashboard: cards corrigidos (nowrap, min-width, layout 3 colunas)
- Botão 'Ver detalhes' nos cards → navega para aba Empresa
- Sparklines: ticker + % 6m na mesma linha (sem ambiguidade)
- Radar: FCF Yield → Margem Líquida (campo disponível no JSON)
- Deduplicação por ticker: manual tem prioridade sobre B3
- Comparativo: filtro de outliers (upside > 500%)
- session_state: empresa pré-selecionada ao clicar em Detalhes
</commit_message>
<xml_diff>
--- a/valuation_output.xlsx
+++ b/valuation_output.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,647 +427,688 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AC7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>CAPEX</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>CASH</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DEBT_LONG</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DEBT_LONG_FIN</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DEBT_SHORT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DEBT_SHORT_FIN</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DEPRECIATION</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>EBT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>FIN_CF</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>FIN_EXPENSE</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>FIN_INCOME</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FIN_INVESTMENTS</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>FIN_INVESTMENTS_LT</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>GA_EXPENSES</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>GROSS_PROFIT</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>INVEST_CF</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>LEASE_LONG</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>LEASE_SHORT</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NET_INCOME</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>OPER_CF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>REVENUE</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SELLING_EXPENSES</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>TAXES</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>TOTAL_ASSETS</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>TOTAL_LIABILITIES</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2018</v>
+      <c r="A2" s="1" t="n">
+        <v>2019</v>
       </c>
       <c r="B2" t="n">
-        <v>429403000</v>
+        <v>677614000</v>
       </c>
       <c r="C2" t="n">
-        <v>2205700000</v>
+        <v>371683000</v>
       </c>
       <c r="D2" t="n">
-        <v>-8500816000</v>
+        <v>-2809622000</v>
       </c>
       <c r="E2" t="n">
-        <v>1723021000</v>
+        <v>11378737000</v>
       </c>
       <c r="F2" t="n">
-        <v>2049093000</v>
+        <v>161000</v>
       </c>
       <c r="G2" t="n">
-        <v>317023000</v>
+        <v>727302000</v>
       </c>
       <c r="H2" t="n">
-        <v>1507031000</v>
+        <v>531000</v>
       </c>
       <c r="I2" t="n">
-        <v>1497542000</v>
+        <v>551000000</v>
       </c>
       <c r="J2" t="n">
-        <v>7853257000</v>
+        <v>1016939000</v>
       </c>
       <c r="K2" t="n">
-        <v>-1446435000</v>
+        <v>183786000</v>
       </c>
       <c r="L2" t="n">
-        <v>-887163000</v>
+        <v>15835269000</v>
       </c>
       <c r="M2" t="n">
-        <v>877674000</v>
+        <v>-1554534000</v>
       </c>
       <c r="N2" t="n">
-        <v>1324188000</v>
+        <v>-1179670000</v>
       </c>
       <c r="O2" t="n">
-        <v>-566631000</v>
+        <v>346517000</v>
       </c>
       <c r="P2" t="n">
-        <v>3469274000</v>
+        <v>453952000</v>
       </c>
       <c r="Q2" t="n">
-        <v>-833290000</v>
+        <v>3254294000</v>
       </c>
       <c r="R2" t="n">
-        <v>2688296000</v>
+        <v>-1702760000</v>
       </c>
       <c r="S2" t="n">
-        <v>1299655000</v>
+        <v>4217572000</v>
       </c>
       <c r="T2" t="n">
-        <v>11970090000</v>
+        <v>21386000</v>
       </c>
       <c r="U2" t="n">
-        <v>-1139413000</v>
+        <v>7504875000</v>
       </c>
       <c r="V2" t="n">
-        <v>-153394000</v>
+        <v>578998000</v>
       </c>
       <c r="W2" t="n">
-        <v>15399850000</v>
+        <v>485176000</v>
       </c>
       <c r="X2" t="n">
-        <v>15399850000</v>
+        <v>419220000</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>7027194000</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>-1536991000</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>58802000</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>34118446000</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>34118446000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2019</v>
+      <c r="A3" s="1" t="n">
+        <v>2020</v>
       </c>
       <c r="B3" t="n">
-        <v>524482000</v>
+        <v>444300000</v>
       </c>
       <c r="C3" t="n">
-        <v>1946044000</v>
+        <v>2205346000</v>
       </c>
       <c r="D3" t="n">
-        <v>-9394166000</v>
+        <v>-1946923000</v>
       </c>
       <c r="E3" t="n">
-        <v>1348599000</v>
+        <v>8084542000</v>
       </c>
       <c r="F3" t="n">
-        <v>936370000</v>
+        <v>817000</v>
       </c>
       <c r="G3" t="n">
-        <v>396783000</v>
+        <v>2169119000</v>
       </c>
       <c r="H3" t="n">
-        <v>1847734000</v>
+        <v>229000</v>
       </c>
       <c r="I3" t="n">
-        <v>1804451000</v>
+        <v>541671000</v>
       </c>
       <c r="J3" t="n">
-        <v>8929990000</v>
+        <v>-3236907000</v>
       </c>
       <c r="K3" t="n">
-        <v>-2115441000</v>
+        <v>-3835601000</v>
       </c>
       <c r="L3" t="n">
-        <v>-960665000</v>
+        <v>14285164000</v>
       </c>
       <c r="M3" t="n">
-        <v>917382000</v>
+        <v>3269197000</v>
       </c>
       <c r="N3" t="n">
-        <v>1444227000</v>
+        <v>-878512000</v>
       </c>
       <c r="O3" t="n">
-        <v>-548407000</v>
+        <v>279818000</v>
       </c>
       <c r="P3" t="n">
-        <v>3953268000</v>
+        <v>1976436000</v>
       </c>
       <c r="Q3" t="n">
-        <v>-59748000</v>
+        <v>2147841000</v>
       </c>
       <c r="R3" t="n">
-        <v>3264910000</v>
+        <v>-1644018000</v>
       </c>
       <c r="S3" t="n">
-        <v>1907853000</v>
+        <v>3322221000</v>
       </c>
       <c r="T3" t="n">
-        <v>13347434000</v>
+        <v>-1533908000</v>
       </c>
       <c r="U3" t="n">
-        <v>-1253165000</v>
+        <v>5171357000</v>
       </c>
       <c r="V3" t="n">
-        <v>-171996000</v>
+        <v>2048808000</v>
       </c>
       <c r="W3" t="n">
-        <v>15687641000</v>
+        <v>-9432181000</v>
       </c>
       <c r="X3" t="n">
-        <v>15687641000</v>
+        <v>256343000</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>5269144000</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>-2293415000</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>209218000</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>30783788000</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>30783788000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2020</v>
+      <c r="A4" s="1" t="n">
+        <v>2021</v>
       </c>
       <c r="B4" t="n">
-        <v>558546000</v>
+        <v>381717000</v>
       </c>
       <c r="C4" t="n">
-        <v>3892140000</v>
+        <v>1601468000</v>
       </c>
       <c r="D4" t="n">
-        <v>-12032050000</v>
+        <v>-1903710000</v>
       </c>
       <c r="E4" t="n">
-        <v>1044296000</v>
+        <v>7635254000</v>
       </c>
       <c r="F4" t="n">
-        <v>642284000</v>
+        <v>651000</v>
       </c>
       <c r="G4" t="n">
-        <v>451359000</v>
+        <v>2258499000</v>
       </c>
       <c r="H4" t="n">
-        <v>2816324000</v>
+        <v>237000</v>
       </c>
       <c r="I4" t="n">
-        <v>2746649000</v>
+        <v>488986000</v>
       </c>
       <c r="J4" t="n">
-        <v>11930298000</v>
+        <v>78404000</v>
       </c>
       <c r="K4" t="n">
-        <v>-2360601000</v>
+        <v>-505368000</v>
       </c>
       <c r="L4" t="n">
-        <v>-1090101000</v>
+        <v>13770664000</v>
       </c>
       <c r="M4" t="n">
-        <v>1020426000</v>
+        <v>-713877000</v>
       </c>
       <c r="N4" t="n">
-        <v>592794000</v>
+        <v>-893598000</v>
       </c>
       <c r="O4" t="n">
-        <v>-654469000</v>
+        <v>309826000</v>
       </c>
       <c r="P4" t="n">
-        <v>5437507000</v>
+        <v>2425201000</v>
       </c>
       <c r="Q4" t="n">
-        <v>207375000</v>
+        <v>1766495000</v>
       </c>
       <c r="R4" t="n">
-        <v>4791914000</v>
+        <v>-1662087000</v>
       </c>
       <c r="S4" t="n">
-        <v>3930032000</v>
+        <v>2874347000</v>
       </c>
       <c r="T4" t="n">
-        <v>17469557000</v>
+        <v>-393601000</v>
       </c>
       <c r="U4" t="n">
-        <v>-1506817000</v>
+        <v>4745154000</v>
       </c>
       <c r="V4" t="n">
-        <v>-350692000</v>
+        <v>2120340000</v>
       </c>
       <c r="W4" t="n">
-        <v>19927896000</v>
+        <v>-974508000</v>
       </c>
       <c r="X4" t="n">
-        <v>19927896000</v>
+        <v>503600000</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>4778057000</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-570753000</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>43845000</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>28512853000</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>28512853000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>2021</v>
+      <c r="A5" s="1" t="n">
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>847344000</v>
+        <v>441569000</v>
       </c>
       <c r="C5" t="n">
-        <v>2714427000</v>
+        <v>121772000</v>
       </c>
       <c r="D5" t="n">
-        <v>-16602381000</v>
+        <v>-1864883000</v>
       </c>
       <c r="E5" t="n">
-        <v>737071000</v>
+        <v>6019508000</v>
       </c>
       <c r="F5" t="n">
-        <v>1052044000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>520178000</v>
+        <v>2184815000</v>
       </c>
       <c r="H5" t="n">
-        <v>4158343000</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>4330036000</v>
+        <v>458040000</v>
       </c>
       <c r="J5" t="n">
-        <v>14010672000</v>
+        <v>303304000</v>
       </c>
       <c r="K5" t="n">
-        <v>-1443405000</v>
+        <v>-592123000</v>
       </c>
       <c r="L5" t="n">
-        <v>-821046000</v>
+        <v>13241388000</v>
       </c>
       <c r="M5" t="n">
-        <v>992739000</v>
+        <v>-2036823000</v>
       </c>
       <c r="N5" t="n">
-        <v>502708000</v>
+        <v>-1405332000</v>
       </c>
       <c r="O5" t="n">
-        <v>-776007000</v>
+        <v>509905000</v>
       </c>
       <c r="P5" t="n">
-        <v>6960957000</v>
+        <v>2007061000</v>
       </c>
       <c r="Q5" t="n">
-        <v>-683870000</v>
+        <v>2033886000</v>
       </c>
       <c r="R5" t="n">
-        <v>7314960000</v>
+        <v>-1709188000</v>
       </c>
       <c r="S5" t="n">
-        <v>939385000</v>
+        <v>3227319000</v>
       </c>
       <c r="T5" t="n">
-        <v>23563338000</v>
+        <v>439780000</v>
       </c>
       <c r="U5" t="n">
-        <v>-1833204000</v>
+        <v>3152882000</v>
       </c>
       <c r="V5" t="n">
-        <v>-672556000</v>
+        <v>2038312000</v>
       </c>
       <c r="W5" t="n">
-        <v>23932787000</v>
+        <v>-1081996000</v>
       </c>
       <c r="X5" t="n">
-        <v>23932787000</v>
+        <v>117347000</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>5092202000</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-548718000</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>51125000</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>26396751000</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>26396751000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>2022</v>
+      <c r="A6" s="1" t="n">
+        <v>2023</v>
       </c>
       <c r="B6" t="n">
-        <v>1174410000</v>
+        <v>456622000</v>
       </c>
       <c r="C6" t="n">
-        <v>4451002000</v>
+        <v>624483000</v>
       </c>
       <c r="D6" t="n">
-        <v>-21209235000</v>
+        <v>-2109212000</v>
       </c>
       <c r="E6" t="n">
-        <v>1151875000</v>
+        <v>6165025000</v>
       </c>
       <c r="F6" t="n">
-        <v>2307817000</v>
+        <v>56959000</v>
       </c>
       <c r="G6" t="n">
-        <v>565557000</v>
+        <v>1610571000</v>
       </c>
       <c r="H6" t="n">
-        <v>5051587000</v>
+        <v>4619000</v>
       </c>
       <c r="I6" t="n">
-        <v>5115642000</v>
+        <v>455741000</v>
       </c>
       <c r="J6" t="n">
-        <v>15248355000</v>
+        <v>732160000</v>
       </c>
       <c r="K6" t="n">
-        <v>191912000</v>
+        <v>-171578000</v>
       </c>
       <c r="L6" t="n">
-        <v>-1133215000</v>
+        <v>12706279000</v>
       </c>
       <c r="M6" t="n">
-        <v>1197270000</v>
+        <v>-682997000</v>
       </c>
       <c r="N6" t="n">
-        <v>531826000</v>
+        <v>-1292099000</v>
       </c>
       <c r="O6" t="n">
-        <v>-872935000</v>
+        <v>388361000</v>
       </c>
       <c r="P6" t="n">
-        <v>8695487000</v>
+        <v>1166805000</v>
       </c>
       <c r="Q6" t="n">
-        <v>-1356262000</v>
+        <v>1338489000</v>
       </c>
       <c r="R6" t="n">
-        <v>8545744000</v>
+        <v>-1766613000</v>
       </c>
       <c r="S6" t="n">
-        <v>2936931000</v>
+        <v>3705586000</v>
       </c>
       <c r="T6" t="n">
-        <v>29904722000</v>
+        <v>505861000</v>
       </c>
       <c r="U6" t="n">
-        <v>-2164802000</v>
+        <v>3422746000</v>
       </c>
       <c r="V6" t="n">
-        <v>-842770000</v>
+        <v>1450226000</v>
       </c>
       <c r="W6" t="n">
-        <v>28134660000</v>
+        <v>-978679000</v>
       </c>
       <c r="X6" t="n">
-        <v>28134660000</v>
+        <v>679847000</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5814798000</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-702994000</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>-295748000</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>25135863000</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>25135863000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>2023</v>
+      <c r="A7" s="1" t="n">
+        <v>2024</v>
       </c>
       <c r="B7" t="n">
-        <v>1658625000</v>
+        <v>410086000</v>
       </c>
       <c r="C7" t="n">
-        <v>6488454000</v>
+        <v>94965000</v>
       </c>
       <c r="D7" t="n">
-        <v>-21702737000</v>
+        <v>-2113100000</v>
       </c>
       <c r="E7" t="n">
-        <v>664737000</v>
+        <v>6028736000</v>
       </c>
       <c r="F7" t="n">
-        <v>2170324000</v>
+        <v>67418000</v>
       </c>
       <c r="G7" t="n">
-        <v>628042000</v>
+        <v>844476000</v>
       </c>
       <c r="H7" t="n">
-        <v>6462125000</v>
+        <v>15270000</v>
       </c>
       <c r="I7" t="n">
-        <v>6590797000</v>
+        <v>457543000</v>
       </c>
       <c r="J7" t="n">
-        <v>17854776000</v>
+        <v>1351968000</v>
       </c>
       <c r="K7" t="n">
-        <v>-2963451000</v>
+        <v>662830000</v>
       </c>
       <c r="L7" t="n">
-        <v>-1424977000</v>
+        <v>13545135000</v>
       </c>
       <c r="M7" t="n">
-        <v>1553649000</v>
+        <v>-1158054000</v>
       </c>
       <c r="N7" t="n">
-        <v>592770000</v>
+        <v>-1245705000</v>
       </c>
       <c r="O7" t="n">
-        <v>-1044888000</v>
+        <v>556567000</v>
       </c>
       <c r="P7" t="n">
-        <v>10800864000</v>
+        <v>1237230000</v>
       </c>
       <c r="Q7" t="n">
-        <v>-1714206000</v>
+        <v>1096485000</v>
       </c>
       <c r="R7" t="n">
-        <v>11735230000</v>
+        <v>-1562979000</v>
       </c>
       <c r="S7" t="n">
-        <v>7021823000</v>
+        <v>4277493000</v>
       </c>
       <c r="T7" t="n">
-        <v>32503601000</v>
+        <v>-238900000</v>
       </c>
       <c r="U7" t="n">
-        <v>-2426459000</v>
+        <v>3272020000</v>
       </c>
       <c r="V7" t="n">
-        <v>-723182000</v>
+        <v>644939000</v>
       </c>
       <c r="W7" t="n">
-        <v>31496270000</v>
+        <v>1986552000</v>
       </c>
       <c r="X7" t="n">
-        <v>31496270000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1850322000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>7347599000</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-25173096000</v>
-      </c>
-      <c r="E8" t="n">
-        <v>744281000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2850956000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>812485000</v>
-      </c>
-      <c r="H8" t="n">
-        <v>7690528000</v>
-      </c>
-      <c r="I8" t="n">
-        <v>7908508000</v>
-      </c>
-      <c r="J8" t="n">
-        <v>23125217000</v>
-      </c>
-      <c r="K8" t="n">
-        <v>-2764198000</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-1724138000</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1942118000</v>
-      </c>
-      <c r="N8" t="n">
-        <v>648477000</v>
-      </c>
-      <c r="O8" t="n">
-        <v>-1299421000</v>
-      </c>
-      <c r="P8" t="n">
-        <v>12813845000</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>-4094629000</v>
-      </c>
-      <c r="R8" t="n">
-        <v>12637526000</v>
-      </c>
-      <c r="S8" t="n">
-        <v>7252269000</v>
-      </c>
-      <c r="T8" t="n">
-        <v>37986941000</v>
-      </c>
-      <c r="U8" t="n">
-        <v>-2987307000</v>
-      </c>
-      <c r="V8" t="n">
-        <v>-1589745000</v>
-      </c>
-      <c r="W8" t="n">
-        <v>41489701000</v>
-      </c>
-      <c r="X8" t="n">
-        <v>41489701000</v>
+        <v>867436000</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>6390593000</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-768095000</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>332091000</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>24200400000</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>24200400000</v>
       </c>
     </row>
   </sheetData>
@@ -1073,132 +1126,132 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>REVENUE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>DEPRECIATION</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>44840015892.66895</v>
+        <v>7096753526.5</v>
       </c>
       <c r="C2" t="n">
-        <v>7508838211.20251</v>
+        <v>1490318240.565</v>
       </c>
       <c r="D2" t="n">
-        <v>1048918358.802241</v>
+        <v>545847295.7543305</v>
       </c>
       <c r="E2" t="n">
-        <v>4955833219.393656</v>
+        <v>983610038.7728999</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="B3" t="n">
-        <v>51977731683.43146</v>
+        <v>7788686995.33375</v>
       </c>
       <c r="C3" t="n">
-        <v>8704108819.461676</v>
+        <v>1635624269.020087</v>
       </c>
       <c r="D3" t="n">
-        <v>1215887102.764428</v>
+        <v>599067407.0903777</v>
       </c>
       <c r="E3" t="n">
-        <v>5744711820.844706</v>
+        <v>1079512017.553258</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="B4" t="n">
-        <v>59148454075.98905</v>
+        <v>8446831046.439452</v>
       </c>
       <c r="C4" t="n">
-        <v>9904906661.104837</v>
+        <v>1773834519.752285</v>
       </c>
       <c r="D4" t="n">
-        <v>1383627952.398197</v>
+        <v>649688602.9895146</v>
       </c>
       <c r="E4" t="n">
-        <v>6537238396.329192</v>
+        <v>1170730783.036508</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2028</v>
       </c>
       <c r="B5" t="n">
-        <v>66053050798.02906</v>
+        <v>9050779466.259872</v>
       </c>
       <c r="C5" t="n">
-        <v>11061139518.45925</v>
+        <v>1900663687.914573</v>
       </c>
       <c r="D5" t="n">
-        <v>1545143467.45085</v>
+        <v>696141338.1032649</v>
       </c>
       <c r="E5" t="n">
-        <v>7300352082.183102</v>
+        <v>1254438034.023618</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2029</v>
       </c>
       <c r="B6" t="n">
-        <v>72361718103.20117</v>
+        <v>9580250065.036076</v>
       </c>
       <c r="C6" t="n">
-        <v>12117578977.27275</v>
+        <v>2011852513.657576</v>
       </c>
       <c r="D6" t="n">
-        <v>1692718726.384966</v>
+        <v>736865606.382306</v>
       </c>
       <c r="E6" t="n">
-        <v>7997602125.000016</v>
+        <v>1327822659.014</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2030</v>
       </c>
       <c r="B7" t="n">
-        <v>77737097770.50198</v>
+        <v>10016151442.99522</v>
       </c>
       <c r="C7" t="n">
-        <v>13017731562.90438</v>
+        <v>2103391803.028996</v>
       </c>
       <c r="D7" t="n">
-        <v>1818462089.903397</v>
+        <v>770392991.472701</v>
       </c>
       <c r="E7" t="n">
-        <v>8591702831.516893</v>
+        <v>1388238589.999137</v>
       </c>
     </row>
   </sheetData>
@@ -1212,704 +1265,786 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z14"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>CAPEX</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>CASH</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>COGS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DEBT_LONG</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DEBT_LONG_FIN</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DEBT_SHORT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DEBT_SHORT_FIN</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DEPRECIATION</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>EBT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>FIN_CF</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>FIN_EXPENSE</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>FIN_INCOME</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FIN_INVESTMENTS</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>FIN_INVESTMENTS_LT</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>GA_EXPENSES</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>GROSS_PROFIT</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>INVEST_CF</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>LEASE_LONG</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>LEASE_SHORT</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NET_INCOME</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>OPER_CF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>REVENUE</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SELLING_EXPENSES</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>TAXES</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>TOTAL_ASSETS</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>TOTAL_LIABILITIES</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2018</v>
+      <c r="A2" s="1" t="n">
+        <v>2019</v>
       </c>
       <c r="B2" t="n">
-        <v>429403000</v>
+        <v>677614000</v>
       </c>
       <c r="C2" t="n">
-        <v>2205700000</v>
+        <v>371683000</v>
       </c>
       <c r="D2" t="n">
-        <v>-8500816000</v>
+        <v>-2809622000</v>
       </c>
       <c r="E2" t="n">
-        <v>1723021000</v>
+        <v>11378737000</v>
       </c>
       <c r="F2" t="n">
-        <v>2049093000</v>
+        <v>161000</v>
       </c>
       <c r="G2" t="n">
-        <v>317023000</v>
+        <v>727302000</v>
       </c>
       <c r="H2" t="n">
-        <v>1507031000</v>
+        <v>531000</v>
       </c>
       <c r="I2" t="n">
-        <v>1497542000</v>
+        <v>551000000</v>
       </c>
       <c r="J2" t="n">
-        <v>7853257000</v>
+        <v>1016939000</v>
       </c>
       <c r="K2" t="n">
-        <v>-1446435000</v>
+        <v>183786000</v>
       </c>
       <c r="L2" t="n">
-        <v>-887163000</v>
+        <v>15835269000</v>
       </c>
       <c r="M2" t="n">
-        <v>877674000</v>
+        <v>-1554534000</v>
       </c>
       <c r="N2" t="n">
-        <v>1324188000</v>
+        <v>-1179670000</v>
       </c>
       <c r="O2" t="n">
-        <v>-566631000</v>
+        <v>346517000</v>
       </c>
       <c r="P2" t="n">
-        <v>3469274000</v>
+        <v>453952000</v>
       </c>
       <c r="Q2" t="n">
-        <v>-833290000</v>
+        <v>3254294000</v>
       </c>
       <c r="R2" t="n">
-        <v>2688296000</v>
+        <v>-1702760000</v>
       </c>
       <c r="S2" t="n">
-        <v>1299655000</v>
+        <v>4217572000</v>
       </c>
       <c r="T2" t="n">
-        <v>11970090000</v>
+        <v>21386000</v>
       </c>
       <c r="U2" t="n">
-        <v>-1139413000</v>
+        <v>7504875000</v>
       </c>
       <c r="V2" t="n">
-        <v>-153394000</v>
+        <v>578998000</v>
       </c>
       <c r="W2" t="n">
-        <v>15399850000</v>
+        <v>485176000</v>
       </c>
       <c r="X2" t="n">
-        <v>15399850000</v>
-      </c>
-      <c r="Y2" t="inlineStr"/>
+        <v>419220000</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>7027194000</v>
+      </c>
       <c r="Z2" t="n">
-        <v>870252000</v>
+        <v>-1536991000</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>58802000</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>34118446000</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>34118446000</v>
+      </c>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="n">
+        <v>-33037000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2019</v>
+      <c r="A3" s="1" t="n">
+        <v>2020</v>
       </c>
       <c r="B3" t="n">
-        <v>524482000</v>
+        <v>444300000</v>
       </c>
       <c r="C3" t="n">
-        <v>1946044000</v>
+        <v>2205346000</v>
       </c>
       <c r="D3" t="n">
-        <v>-9394166000</v>
+        <v>-1946923000</v>
       </c>
       <c r="E3" t="n">
-        <v>1348599000</v>
+        <v>8084542000</v>
       </c>
       <c r="F3" t="n">
-        <v>936370000</v>
+        <v>817000</v>
       </c>
       <c r="G3" t="n">
-        <v>396783000</v>
+        <v>2169119000</v>
       </c>
       <c r="H3" t="n">
-        <v>1847734000</v>
+        <v>229000</v>
       </c>
       <c r="I3" t="n">
-        <v>1804451000</v>
+        <v>541671000</v>
       </c>
       <c r="J3" t="n">
-        <v>8929990000</v>
+        <v>-3236907000</v>
       </c>
       <c r="K3" t="n">
-        <v>-2115441000</v>
+        <v>-3835601000</v>
       </c>
       <c r="L3" t="n">
-        <v>-960665000</v>
+        <v>14285164000</v>
       </c>
       <c r="M3" t="n">
-        <v>917382000</v>
+        <v>3269197000</v>
       </c>
       <c r="N3" t="n">
-        <v>1444227000</v>
+        <v>-878512000</v>
       </c>
       <c r="O3" t="n">
-        <v>-548407000</v>
+        <v>279818000</v>
       </c>
       <c r="P3" t="n">
-        <v>3953268000</v>
+        <v>1976436000</v>
       </c>
       <c r="Q3" t="n">
-        <v>-59748000</v>
+        <v>2147841000</v>
       </c>
       <c r="R3" t="n">
-        <v>3264910000</v>
+        <v>-1644018000</v>
       </c>
       <c r="S3" t="n">
-        <v>1907853000</v>
+        <v>3322221000</v>
       </c>
       <c r="T3" t="n">
-        <v>13347434000</v>
+        <v>-1533908000</v>
       </c>
       <c r="U3" t="n">
-        <v>-1253165000</v>
+        <v>5171357000</v>
       </c>
       <c r="V3" t="n">
-        <v>-171996000</v>
+        <v>2048808000</v>
       </c>
       <c r="W3" t="n">
-        <v>15687641000</v>
+        <v>-9432181000</v>
       </c>
       <c r="X3" t="n">
-        <v>15687641000</v>
-      </c>
-      <c r="Y3" t="inlineStr"/>
+        <v>256343000</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>5269144000</v>
+      </c>
       <c r="Z3" t="n">
-        <v>1383371000</v>
+        <v>-2293415000</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>209218000</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>30783788000</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>30783788000</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="n">
+        <v>-33037000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2020</v>
+      <c r="A4" s="1" t="n">
+        <v>2021</v>
       </c>
       <c r="B4" t="n">
-        <v>558546000</v>
+        <v>381717000</v>
       </c>
       <c r="C4" t="n">
-        <v>3892140000</v>
+        <v>1601468000</v>
       </c>
       <c r="D4" t="n">
-        <v>-12032050000</v>
+        <v>-1903710000</v>
       </c>
       <c r="E4" t="n">
-        <v>1044296000</v>
+        <v>7635254000</v>
       </c>
       <c r="F4" t="n">
-        <v>642284000</v>
+        <v>651000</v>
       </c>
       <c r="G4" t="n">
-        <v>451359000</v>
+        <v>2258499000</v>
       </c>
       <c r="H4" t="n">
-        <v>2816324000</v>
+        <v>237000</v>
       </c>
       <c r="I4" t="n">
-        <v>2746649000</v>
+        <v>488986000</v>
       </c>
       <c r="J4" t="n">
-        <v>11930298000</v>
+        <v>78404000</v>
       </c>
       <c r="K4" t="n">
-        <v>-2360601000</v>
+        <v>-505368000</v>
       </c>
       <c r="L4" t="n">
-        <v>-1090101000</v>
+        <v>13770664000</v>
       </c>
       <c r="M4" t="n">
-        <v>1020426000</v>
+        <v>-713877000</v>
       </c>
       <c r="N4" t="n">
-        <v>592794000</v>
+        <v>-893598000</v>
       </c>
       <c r="O4" t="n">
-        <v>-654469000</v>
+        <v>309826000</v>
       </c>
       <c r="P4" t="n">
-        <v>5437507000</v>
+        <v>2425201000</v>
       </c>
       <c r="Q4" t="n">
-        <v>207375000</v>
+        <v>1766495000</v>
       </c>
       <c r="R4" t="n">
-        <v>4791914000</v>
+        <v>-1662087000</v>
       </c>
       <c r="S4" t="n">
-        <v>3930032000</v>
+        <v>2874347000</v>
       </c>
       <c r="T4" t="n">
-        <v>17469557000</v>
+        <v>-393601000</v>
       </c>
       <c r="U4" t="n">
-        <v>-1506817000</v>
+        <v>4745154000</v>
       </c>
       <c r="V4" t="n">
-        <v>-350692000</v>
+        <v>2120340000</v>
       </c>
       <c r="W4" t="n">
-        <v>19927896000</v>
+        <v>-974508000</v>
       </c>
       <c r="X4" t="n">
-        <v>19927896000</v>
-      </c>
-      <c r="Y4" t="inlineStr"/>
+        <v>503600000</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>4778057000</v>
+      </c>
       <c r="Z4" t="n">
-        <v>3371486000</v>
+        <v>-570753000</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>43845000</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>28512853000</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>28512853000</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="n">
+        <v>121883000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>2021</v>
+      <c r="A5" s="1" t="n">
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>847344000</v>
+        <v>441569000</v>
       </c>
       <c r="C5" t="n">
-        <v>2714427000</v>
+        <v>121772000</v>
       </c>
       <c r="D5" t="n">
-        <v>-16602381000</v>
+        <v>-1864883000</v>
       </c>
       <c r="E5" t="n">
-        <v>737071000</v>
+        <v>6019508000</v>
       </c>
       <c r="F5" t="n">
-        <v>1052044000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>520178000</v>
+        <v>2184815000</v>
       </c>
       <c r="H5" t="n">
-        <v>4158343000</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>4330036000</v>
+        <v>458040000</v>
       </c>
       <c r="J5" t="n">
-        <v>14010672000</v>
+        <v>303304000</v>
       </c>
       <c r="K5" t="n">
-        <v>-1443405000</v>
+        <v>-592123000</v>
       </c>
       <c r="L5" t="n">
-        <v>-821046000</v>
+        <v>13241388000</v>
       </c>
       <c r="M5" t="n">
-        <v>992739000</v>
+        <v>-2036823000</v>
       </c>
       <c r="N5" t="n">
-        <v>502708000</v>
+        <v>-1405332000</v>
       </c>
       <c r="O5" t="n">
-        <v>-776007000</v>
+        <v>509905000</v>
       </c>
       <c r="P5" t="n">
-        <v>6960957000</v>
+        <v>2007061000</v>
       </c>
       <c r="Q5" t="n">
-        <v>-683870000</v>
+        <v>2033886000</v>
       </c>
       <c r="R5" t="n">
-        <v>7314960000</v>
+        <v>-1709188000</v>
       </c>
       <c r="S5" t="n">
-        <v>939385000</v>
+        <v>3227319000</v>
       </c>
       <c r="T5" t="n">
-        <v>23563338000</v>
+        <v>439780000</v>
       </c>
       <c r="U5" t="n">
-        <v>-1833204000</v>
+        <v>3152882000</v>
       </c>
       <c r="V5" t="n">
-        <v>-672556000</v>
+        <v>2038312000</v>
       </c>
       <c r="W5" t="n">
-        <v>23932787000</v>
+        <v>-1081996000</v>
       </c>
       <c r="X5" t="n">
-        <v>23932787000</v>
-      </c>
-      <c r="Y5" t="inlineStr"/>
+        <v>117347000</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>5092202000</v>
+      </c>
       <c r="Z5" t="n">
-        <v>1762521000</v>
+        <v>-548718000</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>51125000</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>26396751000</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>26396751000</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="n">
+        <v>-33037000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>2022</v>
+      <c r="A6" s="1" t="n">
+        <v>2023</v>
       </c>
       <c r="B6" t="n">
-        <v>1174410000</v>
+        <v>456622000</v>
       </c>
       <c r="C6" t="n">
-        <v>4451002000</v>
+        <v>624483000</v>
       </c>
       <c r="D6" t="n">
-        <v>-21209235000</v>
+        <v>-2109212000</v>
       </c>
       <c r="E6" t="n">
-        <v>1151875000</v>
+        <v>6165025000</v>
       </c>
       <c r="F6" t="n">
-        <v>2307817000</v>
+        <v>56959000</v>
       </c>
       <c r="G6" t="n">
-        <v>565557000</v>
+        <v>1610571000</v>
       </c>
       <c r="H6" t="n">
-        <v>5051587000</v>
+        <v>4619000</v>
       </c>
       <c r="I6" t="n">
-        <v>5115642000</v>
+        <v>455741000</v>
       </c>
       <c r="J6" t="n">
-        <v>15248355000</v>
+        <v>732160000</v>
       </c>
       <c r="K6" t="n">
-        <v>191912000</v>
+        <v>-171578000</v>
       </c>
       <c r="L6" t="n">
-        <v>-1133215000</v>
+        <v>12706279000</v>
       </c>
       <c r="M6" t="n">
-        <v>1197270000</v>
+        <v>-682997000</v>
       </c>
       <c r="N6" t="n">
-        <v>531826000</v>
+        <v>-1292099000</v>
       </c>
       <c r="O6" t="n">
-        <v>-872935000</v>
+        <v>388361000</v>
       </c>
       <c r="P6" t="n">
-        <v>8695487000</v>
+        <v>1166805000</v>
       </c>
       <c r="Q6" t="n">
-        <v>-1356262000</v>
+        <v>1338489000</v>
       </c>
       <c r="R6" t="n">
-        <v>8545744000</v>
+        <v>-1766613000</v>
       </c>
       <c r="S6" t="n">
-        <v>2936931000</v>
+        <v>3705586000</v>
       </c>
       <c r="T6" t="n">
-        <v>29904722000</v>
+        <v>505861000</v>
       </c>
       <c r="U6" t="n">
-        <v>-2164802000</v>
+        <v>3422746000</v>
       </c>
       <c r="V6" t="n">
-        <v>-842770000</v>
+        <v>1450226000</v>
       </c>
       <c r="W6" t="n">
-        <v>28134660000</v>
+        <v>-978679000</v>
       </c>
       <c r="X6" t="n">
-        <v>28134660000</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
+        <v>679847000</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5814798000</v>
+      </c>
       <c r="Z6" t="n">
-        <v>1762521000</v>
+        <v>-702994000</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>-295748000</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>25135863000</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>25135863000</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="n">
+        <v>223225000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>2023</v>
+      <c r="A7" s="1" t="n">
+        <v>2024</v>
       </c>
       <c r="B7" t="n">
-        <v>1658625000</v>
+        <v>410086000</v>
       </c>
       <c r="C7" t="n">
-        <v>6488454000</v>
+        <v>94965000</v>
       </c>
       <c r="D7" t="n">
-        <v>-21702737000</v>
+        <v>-2113100000</v>
       </c>
       <c r="E7" t="n">
-        <v>664737000</v>
+        <v>6028736000</v>
       </c>
       <c r="F7" t="n">
-        <v>2170324000</v>
+        <v>67418000</v>
       </c>
       <c r="G7" t="n">
-        <v>628042000</v>
+        <v>844476000</v>
       </c>
       <c r="H7" t="n">
-        <v>6462125000</v>
+        <v>15270000</v>
       </c>
       <c r="I7" t="n">
-        <v>6590797000</v>
+        <v>457543000</v>
       </c>
       <c r="J7" t="n">
-        <v>17854776000</v>
+        <v>1351968000</v>
       </c>
       <c r="K7" t="n">
-        <v>-2963451000</v>
+        <v>662830000</v>
       </c>
       <c r="L7" t="n">
-        <v>-1424977000</v>
+        <v>13545135000</v>
       </c>
       <c r="M7" t="n">
-        <v>1553649000</v>
+        <v>-1158054000</v>
       </c>
       <c r="N7" t="n">
-        <v>592770000</v>
+        <v>-1245705000</v>
       </c>
       <c r="O7" t="n">
-        <v>-1044888000</v>
+        <v>556567000</v>
       </c>
       <c r="P7" t="n">
-        <v>10800864000</v>
+        <v>1237230000</v>
       </c>
       <c r="Q7" t="n">
-        <v>-1714206000</v>
+        <v>1096485000</v>
       </c>
       <c r="R7" t="n">
-        <v>11735230000</v>
+        <v>-1562979000</v>
       </c>
       <c r="S7" t="n">
-        <v>7021823000</v>
+        <v>4277493000</v>
       </c>
       <c r="T7" t="n">
-        <v>32503601000</v>
+        <v>-238900000</v>
       </c>
       <c r="U7" t="n">
-        <v>-2426459000</v>
+        <v>3272020000</v>
       </c>
       <c r="V7" t="n">
-        <v>-723182000</v>
+        <v>644939000</v>
       </c>
       <c r="W7" t="n">
-        <v>31496270000</v>
+        <v>1986552000</v>
       </c>
       <c r="X7" t="n">
-        <v>31496270000</v>
-      </c>
-      <c r="Y7" t="inlineStr"/>
+        <v>867436000</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>6390593000</v>
+      </c>
       <c r="Z7" t="n">
-        <v>5363198000</v>
+        <v>-768095000</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>332091000</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>24200400000</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>24200400000</v>
+      </c>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="n">
+        <v>457350000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1850322000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>7347599000</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-25173096000</v>
-      </c>
-      <c r="E8" t="n">
-        <v>744281000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2850956000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>812485000</v>
-      </c>
-      <c r="H8" t="n">
-        <v>7690528000</v>
-      </c>
+      <c r="A8" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>7908508000</v>
+        <v>545847295.7543305</v>
       </c>
       <c r="J8" t="n">
-        <v>23125217000</v>
-      </c>
-      <c r="K8" t="n">
-        <v>-2764198000</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-1724138000</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1942118000</v>
-      </c>
-      <c r="N8" t="n">
-        <v>648477000</v>
-      </c>
-      <c r="O8" t="n">
-        <v>-1299421000</v>
-      </c>
-      <c r="P8" t="n">
-        <v>12813845000</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>-4094629000</v>
-      </c>
-      <c r="R8" t="n">
-        <v>12637526000</v>
-      </c>
-      <c r="S8" t="n">
-        <v>7252269000</v>
-      </c>
-      <c r="T8" t="n">
-        <v>37986941000</v>
-      </c>
-      <c r="U8" t="n">
-        <v>-2987307000</v>
-      </c>
-      <c r="V8" t="n">
-        <v>-1589745000</v>
-      </c>
-      <c r="W8" t="n">
-        <v>41489701000</v>
-      </c>
-      <c r="X8" t="n">
-        <v>41489701000</v>
-      </c>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="n">
-        <v>5401947000</v>
+        <v>1490318240.565</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="n">
+        <v>7096753526.5</v>
+      </c>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="n">
+        <v>983610038.7728999</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>946775961.0054311</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>2025</v>
+      <c r="A9" s="1" t="n">
+        <v>2026</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>1048918358.802241</v>
-      </c>
-      <c r="H9" t="n">
-        <v>7508838211.20251</v>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>599067407.0903777</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1635624269.020087</v>
+      </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
@@ -1919,37 +2054,42 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="n">
-        <v>44840015892.66895</v>
-      </c>
+      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="n">
-        <v>4955833219.393656</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>4243806832.930941</v>
+        <v>7788686995.33375</v>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="n">
+        <v>1079512017.553258</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>1039086617.203461</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>2026</v>
+      <c r="A10" s="1" t="n">
+        <v>2027</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>1215887102.764428</v>
-      </c>
-      <c r="H10" t="n">
-        <v>8704108819.461676</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>649688602.9895146</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1773834519.752285</v>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
@@ -1959,37 +2099,42 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="n">
-        <v>51977731683.43146</v>
-      </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="n">
-        <v>5744711820.844706</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>4919343771.117205</v>
+        <v>8446831046.439452</v>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="n">
+        <v>1170730783.036508</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>1126889436.357153</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2027</v>
+      <c r="A11" s="1" t="n">
+        <v>2028</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="n">
-        <v>1383627952.398197</v>
-      </c>
-      <c r="H11" t="n">
-        <v>9904906661.104837</v>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>696141338.1032649</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1900663687.914573</v>
+      </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -1999,37 +2144,42 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
-      <c r="T11" t="n">
-        <v>59148454075.98905</v>
-      </c>
+      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="n">
-        <v>6537238396.329192</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>5598004562.84012</v>
+        <v>9050779466.259872</v>
+      </c>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="n">
+        <v>1254438034.023618</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1207462031.05669</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>2028</v>
+      <c r="A12" s="1" t="n">
+        <v>2029</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>1545143467.45085</v>
-      </c>
-      <c r="H12" t="n">
-        <v>11061139518.45925</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>736865606.382306</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2011852513.657576</v>
+      </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -2039,37 +2189,42 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="n">
-        <v>66053050798.02906</v>
-      </c>
+      <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="n">
-        <v>7300352082.183102</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>6251478344.333955</v>
+        <v>9580250065.036076</v>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="n">
+        <v>1327822659.014</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>1278098559.873506</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>2029</v>
+      <c r="A13" s="1" t="n">
+        <v>2030</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>1692718726.384966</v>
-      </c>
-      <c r="H13" t="n">
-        <v>12117578977.27275</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>770392991.472701</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2103391803.028996</v>
+      </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -2079,58 +2234,23 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="n">
-        <v>72361718103.20117</v>
-      </c>
+      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="n">
-        <v>7997602125.000016</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>6848551402.480541</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>1818462089.903397</v>
-      </c>
-      <c r="H14" t="n">
-        <v>13017731562.90438</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="n">
-        <v>77737097770.50198</v>
-      </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="n">
-        <v>8591702831.516893</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>7357295043.791759</v>
+        <v>10016151442.99522</v>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="n">
+        <v>1388238589.999137</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>1336252044.347751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>